<commit_message>
Vestas quote: logo on 1105/1460, call ID on 680CR reflective
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ASRMRMAisA2EYdiMTD5CeW
</commit_message>
<xml_diff>
--- a/Quote - Vestas.xlsx
+++ b/Quote - Vestas.xlsx
@@ -14580,7 +14580,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -14646,7 +14646,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BH01 fleet plate (rear door)</t>
+          <t>BH01 call ID (rear door) - REFLECTIVE</t>
         </is>
       </c>
       <c r="B5" t="n">
@@ -14683,71 +14683,57 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Layout on 1.37m stock</t>
+          <t>Logo - MPI 1105 w/ DOL 1460 (1.37m stock)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Per side: 0.70+0.30 = 1.00m wide &lt;= 1.37m, so logo + plate sit side by side on one row</t>
+          <t>Logo 0.70 x 0.20 -&gt; 0.25m per side incl. margins; 2 sides = 0.50 lm (WORKSHEET!I10), 0.685 m2</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Row height 0.22m + gaps/margins -&gt; 0.25m per side</t>
+          <t>Call ID - 3M 680CR reflective w/ 8519 lustre (1.22m stock, $72/m2)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2 sides x 0.25m = 0.50 lineal m  (entered WORKSHEET!I10, run 1)</t>
+          <t>Both plates 0.30 + 0.30 = 0.60m wide nest on one row, 0.22 + margin = 0.25 lm (WORKSHEET!I18), 0.305 m2</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>Sq m of stock used = 1.37 x 0.5</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr"/>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12">
-        <f>1.37*0.5</f>
-        <v/>
-      </c>
+      <c r="A12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Scale: front door ~0.95m wide in photo -&gt; logo ~0.70m (+/-15%). Plate size is rough.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Stock: MPI 2105 Easy Apply gloss + DOL 2000 clear laminate (flat door panels, per STOCKS from QP); kiss cut on Zund</t>
+          <t>Assumed: 1 vehicle, both sides identical, no rear/tailgate/bonnet graphics, 1 hr install, no freight</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Scale: front door ~0.95m wide in photo -&gt; logo ~0.70m (+/-15%). Plate size is rough.</t>
+          <t>Note: STOCKS tab says DOL 1460 is listed for use with MPI 1005 (old); 1105 normally pairs with 6460. Used 1105/1460 as instructed.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
-        <is>
-          <t>Assumed: 1 vehicle, both sides identical, no rear/tailgate/bonnet graphics, 1 hr install, no freight</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
         <is>
           <t>Master sheet note: WORKSHEET!I9 was hard-coded 0 (kills kiss-cut material); replaced with formula in this copy</t>
         </is>
@@ -17846,7 +17832,7 @@
       </c>
       <c r="B5" s="144" t="inlineStr">
         <is>
-          <t>MPI 2105 EA gloss + DOL 2000 clear (kiss cut)</t>
+          <t>Logo: MPI 1105 w/ DOL 1460; Call ID: 3M 680CR reflective w/ 8519 (kiss cut)</t>
         </is>
       </c>
       <c r="C5" s="147" t="n"/>
@@ -18915,7 +18901,7 @@
       </c>
       <c r="G7" s="47" t="inlineStr">
         <is>
-          <t>MPI 2105 / 2000</t>
+          <t>MPI 1105 w/ 1460</t>
         </is>
       </c>
       <c r="H7" s="45" t="n">
@@ -19256,7 +19242,7 @@
         <v>0</v>
       </c>
       <c r="I18" s="53" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="J18" s="71" t="n">
         <v>0</v>
@@ -19292,7 +19278,7 @@
         <v>1</v>
       </c>
       <c r="I19" s="71" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J19" s="71" t="n">
         <v>1</v>

</xml_diff>